<commit_message>
Daily EOD data and reports for 2026-08-19
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260819.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260819.xlsx
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.375</v>
+        <v>2.38</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.06%</t>
+          <t>1.28%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>166250</v>
+        <v>166600</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1750</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="6">
@@ -569,10 +569,10 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>63.585</v>
+        <v>63.58</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.265</v>
+        <v>-0.27</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -583,10 +583,10 @@
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>703568.03</v>
+        <v>703512.7</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-2932.23</v>
+        <v>-2987.55</v>
       </c>
     </row>
     <row r="8">
@@ -623,10 +623,10 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>160.18</v>
+        <v>160.17</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.45</v>
+        <v>-2.46</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>165.93</v>
+        <v>165.8</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>8.109999999999999</v>
+        <v>7.98</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.14%</t>
+          <t>5.06%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>663720</v>
+        <v>663200</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>32440</v>
+        <v>31920</v>
       </c>
     </row>
     <row r="12">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.605</v>
+        <v>33.6</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.445</v>
+        <v>0.44</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>1.33%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>43283.24</v>
+        <v>43276.8</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>573.16</v>
+        <v>566.72</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1904768.89</v>
+        <v>1904537.13</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>29712.35</v>
+        <v>29480.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>